<commit_message>
Add evaluations single db with middleware
</commit_message>
<xml_diff>
--- a/client-env/profiling/client_profiling_1_db.xlsx
+++ b/client-env/profiling/client_profiling_1_db.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\client-env\profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8024C27D-1895-47C0-971C-BCDFBD475DF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0064E0F8-F35A-478E-A9CB-07A011E36B5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ping Message" sheetId="1" r:id="rId1"/>
@@ -19,12 +19,25 @@
     <sheet name="Get-Range Function" sheetId="4" r:id="rId4"/>
     <sheet name="Delete Function" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="23">
   <si>
     <t>Middleware_Server: 10.0.2.87 (zs07)</t>
   </si>
@@ -32,19 +45,10 @@
     <t>Client: Local</t>
   </si>
   <si>
-    <t>Database_Nodes=5</t>
-  </si>
-  <si>
     <t>Profiling_Iterations=10</t>
   </si>
   <si>
     <t>Client_Instances=1</t>
-  </si>
-  <si>
-    <t>Virtual_Nodes=5</t>
-  </si>
-  <si>
-    <t>Throughput</t>
   </si>
   <si>
     <t>Wall Time: Time taken from sending the response and receiving the response back</t>
@@ -82,6 +86,27 @@
   <si>
     <t>Execution_Time (seconds)</t>
   </si>
+  <si>
+    <t>Database_Nodes=1</t>
+  </si>
+  <si>
+    <t>Virtual_Nodes=0</t>
+  </si>
+  <si>
+    <t>Without_Middleware</t>
+  </si>
+  <si>
+    <t>Difference</t>
+  </si>
+  <si>
+    <t>Key-Value Pairs</t>
+  </si>
+  <si>
+    <t>Difference Per Key</t>
+  </si>
+  <si>
+    <t>Difference Per Key = Difference / Given Key-Value Pairs</t>
+  </si>
 </sst>
 </file>
 
@@ -95,7 +120,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000000E+00"/>
     <numFmt numFmtId="169" formatCode="0.0000000000000000E+00"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,11 +131,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -222,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -234,25 +254,35 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -573,8 +603,9 @@
     <col min="1" max="1" width="39" customWidth="1"/>
     <col min="2" max="2" width="37.85546875" customWidth="1"/>
     <col min="3" max="3" width="33.5703125" customWidth="1"/>
-    <col min="4" max="4" width="23.85546875" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" customWidth="1"/>
     <col min="5" max="5" width="35.5703125" customWidth="1"/>
+    <col min="6" max="6" width="38.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -585,191 +616,227 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="14" t="s">
+      <c r="A6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="12"/>
+      <c r="E6" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="27" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="20">
+      <c r="A7" s="19">
         <v>1</v>
       </c>
-      <c r="B7" s="16">
-        <v>6.0000456869602203E-7</v>
-      </c>
-      <c r="C7" s="16">
-        <v>6.53220003005117E-3</v>
-      </c>
-      <c r="D7" s="8"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15">
+        <v>8.0886000068858196E-3</v>
+      </c>
+      <c r="D7" s="17">
+        <v>2.3041500011458898E-3</v>
+      </c>
+      <c r="E7" s="15">
+        <f>C7-D7</f>
+        <v>5.7844500057399294E-3</v>
+      </c>
+      <c r="F7" s="15">
+        <f>E7/A7</f>
+        <v>5.7844500057399294E-3</v>
+      </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="20">
+      <c r="A8" s="19">
         <v>10</v>
       </c>
-      <c r="B8" s="16">
-        <v>1.20000913739204E-6</v>
-      </c>
-      <c r="C8" s="18">
-        <v>3.0956399976275799E-2</v>
-      </c>
-      <c r="D8" s="9"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="17">
+        <v>3.5332900093635503E-2</v>
+      </c>
+      <c r="D8" s="17">
+        <v>1.8066439998801798E-2</v>
+      </c>
+      <c r="E8" s="15">
+        <f t="shared" ref="E8:E10" si="0">C8-D8</f>
+        <v>1.7266460094833704E-2</v>
+      </c>
+      <c r="F8" s="15">
+        <f t="shared" ref="F8:F10" si="1">E8/A8</f>
+        <v>1.7266460094833703E-3</v>
+      </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="20">
+      <c r="A9" s="19">
         <v>100</v>
       </c>
-      <c r="B9" s="16">
-        <v>5.99992927163839E-6</v>
-      </c>
-      <c r="C9" s="16">
-        <v>0.275612499914132</v>
-      </c>
-      <c r="D9" s="8"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15">
+        <v>0.27911799991852598</v>
+      </c>
+      <c r="D9" s="15">
+        <v>0.17748495001578701</v>
+      </c>
+      <c r="E9" s="15">
+        <f t="shared" si="0"/>
+        <v>0.10163304990273897</v>
+      </c>
+      <c r="F9" s="15">
+        <f t="shared" si="1"/>
+        <v>1.0163304990273897E-3</v>
+      </c>
       <c r="I9" s="7"/>
       <c r="J9" s="7"/>
       <c r="Q9" s="2"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="20">
+      <c r="A10" s="19">
         <v>1000</v>
       </c>
-      <c r="B10" s="16">
-        <v>5.5500073358416503E-5</v>
-      </c>
-      <c r="C10" s="16">
-        <v>2.43718340049963</v>
-      </c>
-      <c r="D10" s="10"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15">
+        <v>2.38097339990781</v>
+      </c>
+      <c r="D10" s="15">
+        <v>1.85243663000874</v>
+      </c>
+      <c r="E10" s="15">
+        <f t="shared" si="0"/>
+        <v>0.52853676989906995</v>
+      </c>
+      <c r="F10" s="15">
+        <f t="shared" si="1"/>
+        <v>5.2853676989906998E-4</v>
+      </c>
       <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="20"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
+      <c r="A11" s="19"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
       <c r="D11" s="8"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="20"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="6"/>
+      <c r="A12" s="19"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="19"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="20"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
+      <c r="A13" s="19"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
       <c r="D13" s="8"/>
-      <c r="E13" s="6"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="19"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" s="20"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
+      <c r="A14" s="19"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
       <c r="D14" s="8"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
     </row>
     <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="21"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="11"/>
+      <c r="A15" s="20"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" s="19"/>
+      <c r="A16" s="18"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
+      <c r="A17" s="18"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
+      <c r="A18" s="18"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
-        <v>9</v>
+      <c r="A19" s="18" t="s">
+        <v>22</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="19">
-        <v>6.6191999940201597E-3</v>
-      </c>
+      <c r="A20" s="18"/>
       <c r="B20" s="4"/>
       <c r="C20" s="3"/>
       <c r="D20" s="6"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="19"/>
+      <c r="A21" s="18"/>
       <c r="B21" s="4"/>
       <c r="C21" s="3"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
+      <c r="A22" s="18"/>
       <c r="B22" s="4"/>
       <c r="C22" s="3"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
+      <c r="A23" s="18"/>
       <c r="B23" s="4"/>
       <c r="C23" s="3"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
+      <c r="A24" s="18"/>
       <c r="B24" s="5"/>
       <c r="C24" s="3"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="19"/>
+      <c r="A25" s="18"/>
       <c r="B25" s="4"/>
       <c r="C25" s="3"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="19"/>
+      <c r="A26" s="18"/>
       <c r="B26" s="4"/>
       <c r="C26" s="3"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>7</v>
-      </c>
-    </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>8</v>
-      </c>
       <c r="B28" s="5"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
-        <v>2.08998244488611E-7</v>
-      </c>
+      <c r="A29" s="14"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" s="4"/>
@@ -977,7 +1044,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{349D7314-AB8E-4AA0-A861-31CE52CA3EE8}">
-  <dimension ref="A1:Q84"/>
+  <dimension ref="A1:R84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39" customWidth="1"/>
@@ -985,9 +1052,11 @@
     <col min="3" max="3" width="33.5703125" customWidth="1"/>
     <col min="4" max="4" width="23.85546875" customWidth="1"/>
     <col min="5" max="5" width="35.5703125" customWidth="1"/>
+    <col min="6" max="6" width="23" customWidth="1"/>
+    <col min="7" max="7" width="26.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -995,201 +1064,245 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
       <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="12" t="s">
+      <c r="F6" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="19">
+        <v>1</v>
+      </c>
+      <c r="C7" s="15"/>
+      <c r="D7" s="17">
+        <v>4.6817200054647401E-3</v>
+      </c>
+      <c r="E7" s="17">
+        <v>2.9214599984697998E-3</v>
+      </c>
+      <c r="F7" s="15">
+        <f>D7-E7</f>
+        <v>1.7602600069949403E-3</v>
+      </c>
+      <c r="G7" s="15">
+        <f>F7/B7</f>
+        <v>1.7602600069949403E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="19">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="20">
-        <v>1</v>
-      </c>
-      <c r="B7" s="16">
-        <v>1.19989272207021E-7</v>
-      </c>
-      <c r="C7" s="18">
-        <v>3.6088000168092499E-3</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="20">
-        <v>10</v>
-      </c>
-      <c r="B8" s="16">
-        <v>1.6000121831893901E-7</v>
-      </c>
-      <c r="C8" s="18">
-        <v>6.8087500054389198E-3</v>
-      </c>
-      <c r="D8" s="22" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="20">
+      <c r="C8" s="15"/>
+      <c r="D8" s="17">
+        <v>5.0182199949631396E-3</v>
+      </c>
+      <c r="E8" s="17">
+        <v>2.9676700010895698E-3</v>
+      </c>
+      <c r="F8" s="15">
+        <f t="shared" ref="F8:F10" si="0">D8-E8</f>
+        <v>2.0505499938735698E-3</v>
+      </c>
+      <c r="G8" s="15">
+        <f t="shared" ref="G8:G10" si="1">F8/B8</f>
+        <v>2.0505499938735697E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="19">
         <v>100</v>
       </c>
-      <c r="B9" s="16">
-        <v>2.2000167518854101E-7</v>
-      </c>
-      <c r="C9" s="16">
-        <v>1.04135300032794E-2</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I9" s="7"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15">
+        <v>1.0857119999127401E-2</v>
+      </c>
+      <c r="E9" s="15">
+        <v>4.7610499896109104E-3</v>
+      </c>
+      <c r="F9" s="15">
+        <f t="shared" si="0"/>
+        <v>6.0960700095164903E-3</v>
+      </c>
+      <c r="G9" s="15">
+        <f t="shared" si="1"/>
+        <v>6.0960700095164904E-5</v>
+      </c>
       <c r="J9" s="7"/>
-      <c r="Q9" s="2"/>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="20">
+      <c r="K9" s="7"/>
+      <c r="R9" s="2"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="19">
         <v>1000</v>
       </c>
-      <c r="B10" s="16">
-        <v>4.9000373110175105E-7</v>
-      </c>
-      <c r="C10" s="16">
-        <v>5.5644339986611099E-2</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="20"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="8"/>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="20"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="6"/>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="20"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="6"/>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" s="20"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="8"/>
-    </row>
-    <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="21"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="11"/>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" s="19"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15">
+        <v>4.4155529997078703E-2</v>
+      </c>
+      <c r="E10" s="15">
+        <v>2.6601759984623601E-2</v>
+      </c>
+      <c r="F10" s="15">
+        <f t="shared" si="0"/>
+        <v>1.7553770012455103E-2</v>
+      </c>
+      <c r="G10" s="15">
+        <f t="shared" si="1"/>
+        <v>1.7553770012455104E-5</v>
+      </c>
+      <c r="I10" s="7"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="8"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="9"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="19"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="8"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="19"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="8"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+    </row>
+    <row r="15" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="18"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
+      <c r="A17" s="18"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
+      <c r="A18" s="18"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
-        <v>9</v>
-      </c>
+      <c r="A19" s="18"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="19">
-        <v>6.6191999940201597E-3</v>
-      </c>
+      <c r="A20" s="18"/>
       <c r="B20" s="4"/>
       <c r="C20" s="3"/>
       <c r="D20" s="6"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="19"/>
+      <c r="A21" s="18"/>
       <c r="B21" s="4"/>
       <c r="C21" s="3"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
+      <c r="A22" s="18"/>
       <c r="B22" s="4"/>
       <c r="C22" s="3"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
+      <c r="A23" s="18"/>
       <c r="B23" s="4"/>
       <c r="C23" s="3"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
+      <c r="A24" s="18"/>
       <c r="B24" s="5"/>
       <c r="C24" s="3"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="19"/>
+      <c r="A25" s="18"/>
       <c r="B25" s="4"/>
       <c r="C25" s="3"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="19"/>
+      <c r="A26" s="18"/>
       <c r="B26" s="4"/>
       <c r="C26" s="3"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>7</v>
-      </c>
-    </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>8</v>
-      </c>
       <c r="B28" s="5"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
-        <v>2.08998244488611E-7</v>
-      </c>
+      <c r="A29" s="14"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" s="4"/>
@@ -1397,7 +1510,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Q84"/>
+  <dimension ref="A1:R84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39" customWidth="1"/>
@@ -1405,9 +1518,11 @@
     <col min="3" max="3" width="33.5703125" customWidth="1"/>
     <col min="4" max="4" width="23.85546875" customWidth="1"/>
     <col min="5" max="5" width="35.5703125" customWidth="1"/>
+    <col min="6" max="6" width="28.5703125" customWidth="1"/>
+    <col min="7" max="7" width="22.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1415,150 +1530,208 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
       <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="12" t="s">
+      <c r="F6" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="19">
+        <v>1</v>
+      </c>
+      <c r="C7" s="15"/>
+      <c r="D7" s="17">
+        <v>3.8862600049469598E-3</v>
+      </c>
+      <c r="E7" s="17">
+        <v>2.4343300028704098E-3</v>
+      </c>
+      <c r="F7" s="15">
+        <f>D7-E7</f>
+        <v>1.45193000207655E-3</v>
+      </c>
+      <c r="G7" s="15">
+        <f>F7/B7</f>
+        <v>1.45193000207655E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="21" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="20">
-        <v>1</v>
-      </c>
-      <c r="B7" s="16">
-        <v>1.20000913739204E-7</v>
-      </c>
-      <c r="C7" s="18">
-        <v>3.5609999787993701E-3</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="20">
+      <c r="B8" s="19">
         <v>10</v>
       </c>
-      <c r="B8" s="16">
-        <v>2.7000205591320898E-7</v>
-      </c>
-      <c r="C8" s="18">
-        <v>5.7667300105094903E-3</v>
-      </c>
-      <c r="D8" s="22" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="20">
+      <c r="C8" s="15"/>
+      <c r="D8" s="17">
+        <v>5.1025999971898196E-3</v>
+      </c>
+      <c r="E8" s="17">
+        <v>2.5533499894663599E-3</v>
+      </c>
+      <c r="F8" s="15">
+        <f t="shared" ref="F8:F10" si="0">D8-E8</f>
+        <v>2.5492500077234598E-3</v>
+      </c>
+      <c r="G8" s="15">
+        <f t="shared" ref="G8:G10" si="1">F8/B8</f>
+        <v>2.5492500077234598E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="19">
         <v>100</v>
       </c>
-      <c r="B9" s="16">
-        <v>3.3000251278281199E-7</v>
-      </c>
-      <c r="C9" s="16">
-        <v>1.1480420012958299E-2</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I9" s="7"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15">
+        <v>9.7233799955574792E-3</v>
+      </c>
+      <c r="E9" s="15">
+        <v>5.1798400003463E-3</v>
+      </c>
+      <c r="F9" s="15">
+        <f t="shared" si="0"/>
+        <v>4.5435399952111792E-3</v>
+      </c>
+      <c r="G9" s="15">
+        <f t="shared" si="1"/>
+        <v>4.5435399952111795E-5</v>
+      </c>
       <c r="J9" s="7"/>
-      <c r="Q9" s="2"/>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="20">
+      <c r="K9" s="7"/>
+      <c r="R9" s="2"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="19">
         <v>1000</v>
       </c>
-      <c r="B10" s="16">
-        <v>0</v>
-      </c>
-      <c r="C10" s="16">
-        <v>5.13304799911566E-2</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="20"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="8"/>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="20"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="6"/>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="20"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="6"/>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" s="20"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="8"/>
-    </row>
-    <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="21"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="11"/>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" s="19"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15">
+        <v>4.6428850002121103E-2</v>
+      </c>
+      <c r="E10" s="15">
+        <v>2.3080520005896599E-2</v>
+      </c>
+      <c r="F10" s="15">
+        <f t="shared" si="0"/>
+        <v>2.3348329996224503E-2</v>
+      </c>
+      <c r="G10" s="15">
+        <f t="shared" si="1"/>
+        <v>2.3348329996224503E-5</v>
+      </c>
+      <c r="I10" s="7"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="8"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="9"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="19"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="8"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="19"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="8"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+    </row>
+    <row r="15" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="18"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
+      <c r="A17" s="18"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
+      <c r="A18" s="18"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
-        <v>9</v>
+      <c r="A19" s="18" t="s">
+        <v>6</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="19">
+      <c r="A20" s="18">
         <v>6.6191999940201597E-3</v>
       </c>
       <c r="B20" s="4"/>
@@ -1566,48 +1739,48 @@
       <c r="D20" s="6"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="19"/>
+      <c r="A21" s="18"/>
       <c r="B21" s="4"/>
       <c r="C21" s="3"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
+      <c r="A22" s="18"/>
       <c r="B22" s="4"/>
       <c r="C22" s="3"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
+      <c r="A23" s="18"/>
       <c r="B23" s="4"/>
       <c r="C23" s="3"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
+      <c r="A24" s="18"/>
       <c r="B24" s="5"/>
       <c r="C24" s="3"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="19"/>
+      <c r="A25" s="18"/>
       <c r="B25" s="4"/>
       <c r="C25" s="3"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="19"/>
+      <c r="A26" s="18"/>
       <c r="B26" s="4"/>
       <c r="C26" s="3"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B28" s="5"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
+      <c r="A29" s="14">
         <v>2.08998244488611E-7</v>
       </c>
     </row>
@@ -1816,7 +1989,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:Q84"/>
+  <dimension ref="A1:R84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39" customWidth="1"/>
@@ -1824,9 +1997,11 @@
     <col min="3" max="3" width="33.5703125" customWidth="1"/>
     <col min="4" max="4" width="23.85546875" customWidth="1"/>
     <col min="5" max="5" width="35.5703125" customWidth="1"/>
+    <col min="6" max="6" width="22.85546875" customWidth="1"/>
+    <col min="7" max="7" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1834,150 +2009,208 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
       <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="12" t="s">
+      <c r="F6" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="19">
+        <v>1</v>
+      </c>
+      <c r="C7" s="15"/>
+      <c r="D7" s="17">
+        <v>4.0637300058733597E-3</v>
+      </c>
+      <c r="E7" s="17">
+        <v>2.9287799960002301E-3</v>
+      </c>
+      <c r="F7" s="15">
+        <f>D7-E7</f>
+        <v>1.1349500098731297E-3</v>
+      </c>
+      <c r="G7" s="15">
+        <f>F7/B7</f>
+        <v>1.1349500098731297E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="19">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="20">
-        <v>1</v>
-      </c>
-      <c r="B7" s="16">
-        <v>0</v>
-      </c>
-      <c r="C7" s="18">
-        <v>3.43204998644068E-3</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="20">
-        <v>10</v>
-      </c>
-      <c r="B8" s="16">
-        <v>0</v>
-      </c>
-      <c r="C8" s="18">
-        <v>5.06252999491989E-3</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="20">
+      <c r="C8" s="15"/>
+      <c r="D8" s="17">
+        <v>4.5849200017983004E-3</v>
+      </c>
+      <c r="E8" s="17">
+        <v>3.8782599964178998E-3</v>
+      </c>
+      <c r="F8" s="15">
+        <f t="shared" ref="F8:F10" si="0">D8-E8</f>
+        <v>7.0666000538040057E-4</v>
+      </c>
+      <c r="G8" s="15">
+        <f t="shared" ref="G8:G10" si="1">F8/B8</f>
+        <v>7.0666000538040062E-5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="19">
         <v>100</v>
       </c>
-      <c r="B9" s="16">
-        <v>0</v>
-      </c>
-      <c r="C9" s="16">
-        <v>9.98640999896451E-3</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="I9" s="7"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15">
+        <v>9.0460499981418196E-3</v>
+      </c>
+      <c r="E9" s="15">
+        <v>5.8791999937966403E-3</v>
+      </c>
+      <c r="F9" s="15">
+        <f t="shared" si="0"/>
+        <v>3.1668500043451793E-3</v>
+      </c>
+      <c r="G9" s="15">
+        <f t="shared" si="1"/>
+        <v>3.1668500043451791E-5</v>
+      </c>
       <c r="J9" s="7"/>
-      <c r="Q9" s="2"/>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="20">
+      <c r="K9" s="7"/>
+      <c r="R9" s="2"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="19">
         <v>1000</v>
       </c>
-      <c r="B10" s="16">
-        <v>0</v>
-      </c>
-      <c r="C10" s="16">
-        <v>4.8389560007490201E-2</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="20"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="8"/>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="20"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="6"/>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="20"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="6"/>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" s="20"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="8"/>
-    </row>
-    <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="21"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="11"/>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" s="19"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15">
+        <v>4.1607220002333599E-2</v>
+      </c>
+      <c r="E10" s="15">
+        <v>2.5481500010937401E-2</v>
+      </c>
+      <c r="F10" s="15">
+        <f t="shared" si="0"/>
+        <v>1.6125719991396198E-2</v>
+      </c>
+      <c r="G10" s="15">
+        <f t="shared" si="1"/>
+        <v>1.6125719991396197E-5</v>
+      </c>
+      <c r="I10" s="7"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="8"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="9"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="19"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="8"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="19"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="8"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+    </row>
+    <row r="15" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="18"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
+      <c r="A17" s="18"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
+      <c r="A18" s="18"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
-        <v>9</v>
+      <c r="A19" s="18" t="s">
+        <v>6</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="19">
+      <c r="A20" s="18">
         <v>6.6191999940201597E-3</v>
       </c>
       <c r="B20" s="4"/>
@@ -1985,48 +2218,48 @@
       <c r="D20" s="6"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="19"/>
+      <c r="A21" s="18"/>
       <c r="B21" s="4"/>
       <c r="C21" s="3"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
+      <c r="A22" s="18"/>
       <c r="B22" s="4"/>
       <c r="C22" s="3"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
+      <c r="A23" s="18"/>
       <c r="B23" s="4"/>
       <c r="C23" s="3"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
+      <c r="A24" s="18"/>
       <c r="B24" s="5"/>
       <c r="C24" s="3"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="19"/>
+      <c r="A25" s="18"/>
       <c r="B25" s="4"/>
       <c r="C25" s="3"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="19"/>
+      <c r="A26" s="18"/>
       <c r="B26" s="4"/>
       <c r="C26" s="3"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B28" s="5"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
+      <c r="A29" s="14">
         <v>2.08998244488611E-7</v>
       </c>
     </row>
@@ -2235,7 +2468,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:Q84"/>
+  <dimension ref="A1:R84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39" customWidth="1"/>
@@ -2243,9 +2476,11 @@
     <col min="3" max="3" width="33.5703125" customWidth="1"/>
     <col min="4" max="4" width="23.85546875" customWidth="1"/>
     <col min="5" max="5" width="35.5703125" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
+    <col min="7" max="7" width="28.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2253,201 +2488,245 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
       <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="12" t="s">
+      <c r="F6" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="19">
+        <v>1</v>
+      </c>
+      <c r="C7" s="15"/>
+      <c r="D7" s="17">
+        <v>4.6853900043061E-3</v>
+      </c>
+      <c r="E7" s="17">
+        <v>2.2126199910417199E-3</v>
+      </c>
+      <c r="F7" s="15">
+        <f>D7-E7</f>
+        <v>2.47277001326438E-3</v>
+      </c>
+      <c r="G7" s="15">
+        <f>F7/B7</f>
+        <v>2.47277001326438E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="19">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="20">
-        <v>1</v>
-      </c>
-      <c r="B7" s="16">
-        <v>0</v>
-      </c>
-      <c r="C7" s="18">
-        <v>3.3188699977472402E-3</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="20">
-        <v>10</v>
-      </c>
-      <c r="B8" s="16">
-        <v>0</v>
-      </c>
-      <c r="C8" s="18">
-        <v>6.1808899976313102E-3</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="20">
+      <c r="C8" s="15"/>
+      <c r="D8" s="17">
+        <v>4.8281599942129102E-3</v>
+      </c>
+      <c r="E8" s="17">
+        <v>2.9057799984002399E-3</v>
+      </c>
+      <c r="F8" s="15">
+        <f t="shared" ref="F8:F10" si="0">D8-E8</f>
+        <v>1.9223799958126703E-3</v>
+      </c>
+      <c r="G8" s="15">
+        <f t="shared" ref="G8:G10" si="1">F8/B8</f>
+        <v>1.9223799958126704E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="19">
         <v>100</v>
       </c>
-      <c r="B9" s="16">
-        <v>0</v>
-      </c>
-      <c r="C9" s="16">
-        <v>9.4462000066414392E-3</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" s="7"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15">
+        <v>8.0048400035593603E-3</v>
+      </c>
+      <c r="E9" s="15">
+        <v>4.2851400037761701E-3</v>
+      </c>
+      <c r="F9" s="15">
+        <f t="shared" si="0"/>
+        <v>3.7196999997831902E-3</v>
+      </c>
+      <c r="G9" s="15">
+        <f t="shared" si="1"/>
+        <v>3.7196999997831904E-5</v>
+      </c>
       <c r="J9" s="7"/>
-      <c r="Q9" s="2"/>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="20">
+      <c r="K9" s="7"/>
+      <c r="R9" s="2"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="19">
         <v>1000</v>
       </c>
-      <c r="B10" s="16">
-        <v>0</v>
-      </c>
-      <c r="C10" s="16">
-        <v>3.7843140005134002E-2</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="20"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="8"/>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="20"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="6"/>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="20"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="6"/>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" s="20"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="8"/>
-    </row>
-    <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="21"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="11"/>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" s="19"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15">
+        <v>3.0715280002914298E-2</v>
+      </c>
+      <c r="E10" s="15">
+        <v>1.4965470001334301E-2</v>
+      </c>
+      <c r="F10" s="15">
+        <f t="shared" si="0"/>
+        <v>1.5749810001579996E-2</v>
+      </c>
+      <c r="G10" s="15">
+        <f t="shared" si="1"/>
+        <v>1.5749810001579995E-5</v>
+      </c>
+      <c r="I10" s="7"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="8"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="9"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="19"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="8"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="19"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="8"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+    </row>
+    <row r="15" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="18"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
+      <c r="A17" s="18"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
+      <c r="A18" s="18"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
-        <v>9</v>
-      </c>
+      <c r="A19" s="18"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="19">
-        <v>6.6191999940201597E-3</v>
-      </c>
+      <c r="A20" s="18"/>
       <c r="B20" s="4"/>
       <c r="C20" s="3"/>
       <c r="D20" s="6"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="19"/>
+      <c r="A21" s="18"/>
       <c r="B21" s="4"/>
       <c r="C21" s="3"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
+      <c r="A22" s="18"/>
       <c r="B22" s="4"/>
       <c r="C22" s="3"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
+      <c r="A23" s="18"/>
       <c r="B23" s="4"/>
       <c r="C23" s="3"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
+      <c r="A24" s="18"/>
       <c r="B24" s="5"/>
       <c r="C24" s="3"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="19"/>
+      <c r="A25" s="18"/>
       <c r="B25" s="4"/>
       <c r="C25" s="3"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="19"/>
+      <c r="A26" s="18"/>
       <c r="B26" s="4"/>
       <c r="C26" s="3"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>7</v>
-      </c>
-    </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>8</v>
-      </c>
       <c r="B28" s="5"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
-        <v>2.08998244488611E-7</v>
-      </c>
+      <c r="A29" s="14"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" s="4"/>

</xml_diff>